<commit_message>
Update robot selector model codes
</commit_message>
<xml_diff>
--- a/InoRobotSelect/Robot_model.xlsx
+++ b/InoRobotSelect/Robot_model.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCARA Robot" sheetId="1" r:id="R5a968800b2234a67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6-Axis Robot" sheetId="2" r:id="R1b8613d84c45411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessories" sheetId="3" r:id="Raae3927270f8491e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expansion Card" sheetId="4" r:id="R2ae65bfc7a4f4640"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCARA Robot" sheetId="1" r:id="R7fee3f2713174efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6-Axis Robot" sheetId="2" r:id="R03ba95a2e12d49d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessories" sheetId="3" r:id="Raeda937511494918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expansion Card" sheetId="4" r:id="Ra85408ed6f6d446e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,9 +201,6 @@
     <x:t xml:space="preserve">IR-GS60-120Z40S-INT</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">01741367*M00002</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">01741340*M00003</x:t>
   </x:si>
   <x:si>
@@ -349,16 +346,10 @@
     <x:t xml:space="preserve">01741086*M00005</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">IR-R15H-145S-INT</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">IR-R16-210S-INT</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">01741090</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">IR-R20H-120S-INT</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">IR-R25-178S-INT</x:t>
@@ -2370,8 +2361,8 @@
       <x:c r="B66" s="38" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C66" s="17" t="s">
-        <x:v>14</x:v>
+      <x:c r="C66" s="17" t="str">
+        <x:v>01741436*M00002</x:v>
       </x:c>
       <x:c r="D66" s="18" t="s">
         <x:v>36</x:v>
@@ -3039,11 +3030,9 @@
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="39"/>
-      <x:c r="B107" s="42" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="C107" s="19" t="s">
-        <x:v>53</x:v>
+      <x:c r="B107" s="42"/>
+      <x:c r="C107" s="19" t="str">
+        <x:v>01741367*M00002</x:v>
       </x:c>
       <x:c r="D107" s="14" t="s">
         <x:v>38</x:v>
@@ -3055,9 +3044,7 @@
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="39"/>
-      <x:c r="B108" s="42" t="s">
-        <x:v>52</x:v>
-      </x:c>
+      <x:c r="B108" s="42"/>
       <x:c r="C108" s="17" t="s">
         <x:v>14</x:v>
       </x:c>
@@ -3071,11 +3058,9 @@
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="39"/>
-      <x:c r="B109" s="42" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="C109" s="17" t="s">
-        <x:v>14</x:v>
+      <x:c r="B109" s="42"/>
+      <x:c r="C109" s="17" t="str">
+        <x:v>01741367*M00003</x:v>
       </x:c>
       <x:c r="D109" s="18" t="s">
         <x:v>18</x:v>
@@ -3087,9 +3072,7 @@
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="39"/>
-      <x:c r="B110" s="42" t="s">
-        <x:v>52</x:v>
-      </x:c>
+      <x:c r="B110" s="42"/>
       <x:c r="C110" s="17" t="s">
         <x:v>14</x:v>
       </x:c>
@@ -3103,9 +3086,7 @@
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="39"/>
-      <x:c r="B111" s="42" t="s">
-        <x:v>52</x:v>
-      </x:c>
+      <x:c r="B111" s="42"/>
       <x:c r="C111" s="17" t="s">
         <x:v>14</x:v>
       </x:c>
@@ -3119,9 +3100,7 @@
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="39"/>
-      <x:c r="B112" s="42" t="s">
-        <x:v>52</x:v>
-      </x:c>
+      <x:c r="B112" s="42"/>
       <x:c r="C112" s="17" t="s">
         <x:v>14</x:v>
       </x:c>
@@ -3135,9 +3114,7 @@
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="40"/>
-      <x:c r="B113" s="43" t="s">
-        <x:v>52</x:v>
-      </x:c>
+      <x:c r="B113" s="43"/>
       <x:c r="C113" s="17" t="s">
         <x:v>14</x:v>
       </x:c>
@@ -3181,7 +3158,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="C115" s="15" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D115" s="14" t="s">
         <x:v>38</x:v>
@@ -3289,13 +3266,13 @@
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="38" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B122" s="44" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B122" s="44" t="s">
+      <x:c r="C122" s="15" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="C122" s="15" t="s">
-        <x:v>57</x:v>
       </x:c>
       <x:c r="D122" s="14" t="s">
         <x:v>12</x:v>
@@ -3413,13 +3390,13 @@
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="38" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B130" s="44" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="C130" s="15" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="C130" s="15" t="s">
-        <x:v>59</x:v>
       </x:c>
       <x:c r="D130" s="14" t="s">
         <x:v>12</x:v>
@@ -3537,10 +3514,10 @@
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="48" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B139" s="38" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="B139" s="38" t="s">
-        <x:v>61</x:v>
       </x:c>
       <x:c r="C139" s="17" t="s">
         <x:v>14</x:v>
@@ -3561,7 +3538,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I139" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -3671,10 +3648,10 @@
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B147" s="44" t="s">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C147" s="17" t="s">
         <x:v>14</x:v>
@@ -3695,7 +3672,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I147" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -3805,10 +3782,10 @@
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B155" s="44" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C155" s="17" t="s">
         <x:v>14</x:v>
@@ -3829,7 +3806,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I155" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
@@ -3939,10 +3916,10 @@
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B163" s="44" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C163" s="17" t="s">
         <x:v>14</x:v>
@@ -3963,7 +3940,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I163" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="164">
@@ -4073,10 +4050,10 @@
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B171" s="44" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C171" s="17" t="s">
         <x:v>14</x:v>
@@ -4097,7 +4074,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I171" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -4207,10 +4184,10 @@
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B179" s="44" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C179" s="17" t="s">
         <x:v>14</x:v>
@@ -4231,7 +4208,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I179" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="180">
@@ -4341,10 +4318,10 @@
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B187" s="44" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C187" s="17" t="s">
         <x:v>14</x:v>
@@ -4365,7 +4342,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I187" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="188">
@@ -4475,10 +4452,10 @@
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B195" s="38" t="s">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C195" s="17" t="s">
         <x:v>14</x:v>
@@ -4499,7 +4476,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I195" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="196">
@@ -4609,10 +4586,10 @@
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B203" s="38" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C203" s="17" t="s">
         <x:v>14</x:v>
@@ -4633,7 +4610,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I203" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="204">
@@ -4743,10 +4720,10 @@
     </x:row>
     <x:row r="211">
       <x:c r="A211" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B211" s="38" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C211" s="17" t="s">
         <x:v>14</x:v>
@@ -4767,7 +4744,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I211" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="212">
@@ -4877,10 +4854,10 @@
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B219" s="45" t="s">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C219" s="17" t="s">
         <x:v>14</x:v>
@@ -4901,7 +4878,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I219" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="220">
@@ -5011,10 +4988,10 @@
     </x:row>
     <x:row r="227">
       <x:c r="A227" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B227" s="45" t="s">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C227" s="17" t="s">
         <x:v>14</x:v>
@@ -5035,7 +5012,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I227" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="228">
@@ -5159,10 +5136,10 @@
     </x:row>
     <x:row r="235">
       <x:c r="A235" s="48" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B235" s="45" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C235" s="17" t="s">
         <x:v>14</x:v>
@@ -5183,7 +5160,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I235" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="236">
@@ -5307,10 +5284,10 @@
     </x:row>
     <x:row r="244">
       <x:c r="A244" s="38" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B244" s="38" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="B244" s="38" t="s">
-        <x:v>76</x:v>
       </x:c>
       <x:c r="C244" s="17" t="s">
         <x:v>14</x:v>
@@ -5331,7 +5308,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I244" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="245">
@@ -5441,10 +5418,10 @@
     </x:row>
     <x:row r="252">
       <x:c r="A252" s="38" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B252" s="44" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C252" s="17" t="s">
         <x:v>14</x:v>
@@ -5465,7 +5442,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I252" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="253">
@@ -5575,10 +5552,10 @@
     </x:row>
     <x:row r="260">
       <x:c r="A260" s="38" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B260" s="44" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C260" s="17" t="s">
         <x:v>14</x:v>
@@ -5599,7 +5576,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I260" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="261">
@@ -5709,10 +5686,10 @@
     </x:row>
     <x:row r="268">
       <x:c r="A268" s="38" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B268" s="44" t="s">
-        <x:v>80</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C268" s="17" t="s">
         <x:v>14</x:v>
@@ -5733,7 +5710,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I268" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="269">
@@ -5843,10 +5820,10 @@
     </x:row>
     <x:row r="276">
       <x:c r="A276" s="38" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B276" s="44" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C276" s="17" t="s">
         <x:v>14</x:v>
@@ -5867,7 +5844,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I276" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="277">
@@ -5977,10 +5954,10 @@
     </x:row>
     <x:row r="284">
       <x:c r="A284" s="38" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B284" s="44" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C284" s="17" t="s">
         <x:v>14</x:v>
@@ -6001,7 +5978,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I284" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="285">
@@ -6111,10 +6088,10 @@
     </x:row>
     <x:row r="292">
       <x:c r="A292" s="38" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B292" s="44" t="s">
-        <x:v>83</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="C292" s="17" t="s">
         <x:v>14</x:v>
@@ -6135,7 +6112,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I292" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="293">
@@ -6537,10 +6514,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="38" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B2" s="50" t="s">
         <x:v>84</x:v>
-      </x:c>
-      <x:c r="B2" s="50" t="s">
-        <x:v>85</x:v>
       </x:c>
       <x:c r="C2" s="17" t="s">
         <x:v>14</x:v>
@@ -6565,7 +6542,7 @@
       <x:c r="A3" s="39"/>
       <x:c r="B3" s="51"/>
       <x:c r="C3" s="15" t="s">
-        <x:v>86</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
         <x:v>38</x:v>
@@ -6661,10 +6638,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B10" s="50" t="s">
-        <x:v>87</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C10" s="17" t="s">
         <x:v>14</x:v>
@@ -6685,14 +6662,14 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I10" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="39"/>
       <x:c r="B11" s="51"/>
       <x:c r="C11" s="15" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="D11" s="14" t="s">
         <x:v>38</x:v>
@@ -6795,10 +6772,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B18" s="50" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="C18" s="17" t="s">
         <x:v>14</x:v>
@@ -6819,14 +6796,14 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I18" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="39"/>
       <x:c r="B19" s="51"/>
       <x:c r="C19" s="34" t="s">
-        <x:v>90</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D19" s="14" t="s">
         <x:v>38</x:v>
@@ -6929,13 +6906,13 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B26" s="53" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C26" s="31" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="C26" s="31" t="s">
-        <x:v>92</x:v>
       </x:c>
       <x:c r="D26" s="33" t="s">
         <x:v>36</x:v>
@@ -6953,14 +6930,14 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I26" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="39"/>
       <x:c r="B27" s="53"/>
       <x:c r="C27" s="34" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D27" s="14" t="s">
         <x:v>38</x:v>
@@ -7063,10 +7040,10 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B34" s="50" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C34" s="17" t="s">
         <x:v>14</x:v>
@@ -7091,7 +7068,7 @@
       <x:c r="A35" s="39"/>
       <x:c r="B35" s="51"/>
       <x:c r="C35" s="15" t="s">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D35" s="14" t="s">
         <x:v>38</x:v>
@@ -7187,10 +7164,10 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B42" s="50" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C42" s="17" t="s">
         <x:v>14</x:v>
@@ -7215,7 +7192,7 @@
       <x:c r="A43" s="39"/>
       <x:c r="B43" s="51"/>
       <x:c r="C43" s="15" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D43" s="14" t="s">
         <x:v>38</x:v>
@@ -7311,10 +7288,10 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B50" s="50" t="s">
-        <x:v>98</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C50" s="17" t="s">
         <x:v>14</x:v>
@@ -7335,14 +7312,14 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I50" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="39"/>
       <x:c r="B51" s="51"/>
       <x:c r="C51" s="34" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D51" s="14" t="s">
         <x:v>38</x:v>
@@ -7445,10 +7422,10 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B58" s="50" t="s">
-        <x:v>100</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C58" s="17" t="str">
         <x:v>01741086*M00008</x:v>
@@ -7473,7 +7450,7 @@
       <x:c r="A59" s="39"/>
       <x:c r="B59" s="51"/>
       <x:c r="C59" s="34" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D59" s="14" t="s">
         <x:v>38</x:v>
@@ -7569,10 +7546,10 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="38" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="B66" s="50" t="s">
-        <x:v>102</x:v>
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B66" s="50" t="str">
+        <x:v>IR-R15H-145S-K-INT</x:v>
       </x:c>
       <x:c r="C66" s="17" t="s">
         <x:v>14</x:v>
@@ -7593,7 +7570,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I66" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -7703,10 +7680,10 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B74" s="53" t="s">
-        <x:v>103</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C74" s="7"/>
       <x:c r="D74" s="16" t="s">
@@ -7729,7 +7706,7 @@
       <x:c r="A75" s="39"/>
       <x:c r="B75" s="53"/>
       <x:c r="C75" s="35" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D75" s="14" t="s">
         <x:v>38</x:v>
@@ -7825,10 +7802,10 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="38" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="B82" s="50" t="s">
-        <x:v>105</x:v>
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B82" s="50" t="str">
+        <x:v>IR-R20H-120S-K-INT</x:v>
       </x:c>
       <x:c r="C82" s="7"/>
       <x:c r="D82" s="16" t="s">
@@ -7847,7 +7824,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="I82" s="49" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -7957,13 +7934,13 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="38" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B90" s="53" t="s">
-        <x:v>106</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="C90" s="37" t="s">
-        <x:v>107</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D90" s="33" t="s">
         <x:v>36</x:v>
@@ -7985,7 +7962,7 @@
       <x:c r="A91" s="39"/>
       <x:c r="B91" s="53"/>
       <x:c r="C91" s="36" t="s">
-        <x:v>108</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D91" s="14" t="s">
         <x:v>38</x:v>
@@ -8041,7 +8018,7 @@
       <x:c r="A95" s="39"/>
       <x:c r="B95" s="53"/>
       <x:c r="C95" s="37" t="s">
-        <x:v>109</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D95" s="32" t="s">
         <x:v>20</x:v>
@@ -8179,130 +8156,130 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1" ht="21" customHeight="1">
       <x:c r="A1" s="4" t="s">
-        <x:v>110</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B1" s="4" t="s">
-        <x:v>111</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C1" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D1" s="5" t="s">
-        <x:v>112</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="E1" s="5" t="s">
-        <x:v>113</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="F1" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A2" s="13" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B2" s="13" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="D2" s="25" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="B2" s="13" t="s">
+      <x:c r="E2" s="2" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="C2" s="2" t="s">
+      <x:c r="F2" s="3" t="s">
         <x:v>117</x:v>
-      </x:c>
-      <x:c r="D2" s="25" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="E2" s="2" t="s">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="F2" s="3" t="s">
-        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A3" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B3" s="13" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C3" s="2">
         <x:v>15050817</x:v>
       </x:c>
       <x:c r="D3" s="25" t="s">
-        <x:v>121</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
-        <x:v>122</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
-        <x:v>123</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A4" s="13" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="D4" s="25" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="B4" s="13" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="C4" s="2" t="s">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="D4" s="25" t="s">
-        <x:v>118</x:v>
-      </x:c>
       <x:c r="E4" s="2" t="s">
-        <x:v>122</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
-        <x:v>123</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A5" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B5" s="13" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="D5" s="25" t="s">
-        <x:v>121</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="E5" s="2" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>127</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A6" s="13" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="C6" s="3" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="D6" s="12" t="s">
-        <x:v>118</x:v>
-      </x:c>
       <x:c r="E6" s="2" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
-        <x:v>127</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A7" s="13" t="s">
-        <x:v>129</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B7" s="13" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C7" s="2">
         <x:v>15050930</x:v>
@@ -8311,690 +8288,690 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E7" s="2" t="s">
-        <x:v>130</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
-        <x:v>131</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A8" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B8" s="13" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
-        <x:v>132</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D8" s="26" t="s">
-        <x:v>133</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E8" s="2" t="s">
-        <x:v>130</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
-        <x:v>134</x:v>
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A9" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B9" s="13" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D9" s="26" t="s">
         <x:v>36</x:v>
       </x:c>
       <x:c r="E9" s="2" t="s">
-        <x:v>130</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
-        <x:v>134</x:v>
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A10" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B10" s="13" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D10" s="26" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="E10" s="2" t="s">
-        <x:v>130</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
-        <x:v>134</x:v>
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A11" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B11" s="13" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="D11" s="25" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="E11" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="12" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A12" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B12" s="13" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="s">
         <x:v>137</x:v>
-      </x:c>
-      <x:c r="C12" s="2" t="s">
-        <x:v>140</x:v>
       </x:c>
       <x:c r="D12" s="25" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E12" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="13" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A13" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B13" s="13" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C13" s="2" t="s">
-        <x:v>141</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="D13" s="25" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E13" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
-        <x:v>142</x:v>
+        <x:v>139</x:v>
       </x:c>
     </x:row>
     <x:row r="14" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A14" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B14" s="13" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C14" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="D14" s="25" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="E14" s="2" t="s">
-        <x:v>144</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A15" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B15" s="13" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C15" s="2" t="s">
-        <x:v>146</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="D15" s="25" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="E15" s="2" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="F15" s="3" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="F15" s="3" t="s">
-        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A16" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B16" s="13" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C16" s="2" t="s">
-        <x:v>148</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D16" s="25" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E16" s="2" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="F16" s="3" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="F16" s="3" t="s">
-        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A17" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B17" s="13" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C17" s="2" t="s">
-        <x:v>149</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D17" s="25" t="s">
         <x:v>18</x:v>
       </x:c>
       <x:c r="E17" s="2" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="F17" s="3" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="F17" s="3" t="s">
-        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="16.5" customHeight="1">
       <x:c r="A18" s="3" t="s">
-        <x:v>129</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
-        <x:v>150</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C18" s="2" t="s">
-        <x:v>151</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D18" s="26" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E18" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
-        <x:v>152</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="16.5" customHeight="1">
       <x:c r="A19" s="3" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="B19" s="3" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="F19" s="3" t="s">
         <x:v>153</x:v>
-      </x:c>
-      <x:c r="B19" s="3" t="s">
-        <x:v>154</x:v>
-      </x:c>
-      <x:c r="C19" s="2" t="s">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="D19" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E19" s="2" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="F19" s="3" t="s">
-        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="16.5" customHeight="1">
       <x:c r="A20" s="3" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="B20" s="3" t="s">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="D20" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="B20" s="3" t="s">
+      <x:c r="F20" s="3" t="s">
         <x:v>158</x:v>
-      </x:c>
-      <x:c r="C20" s="2" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="D20" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E20" s="2" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="F20" s="3" t="s">
-        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
       <x:c r="A21" s="3" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="B21" s="3" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="D21" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="B21" s="3" t="s">
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="C21" s="2" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="D21" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E21" s="2" t="s">
-        <x:v>160</x:v>
-      </x:c>
       <x:c r="F21" s="3" t="s">
-        <x:v>161</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="16.5" customHeight="1">
       <x:c r="A22" s="3" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="B22" s="3" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="D22" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="B22" s="3" t="s">
-        <x:v>164</x:v>
-      </x:c>
-      <x:c r="C22" s="2" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="D22" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E22" s="2" t="s">
-        <x:v>160</x:v>
-      </x:c>
       <x:c r="F22" s="3" t="s">
-        <x:v>161</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="16.5" customHeight="1">
       <x:c r="A23" s="3" t="s">
-        <x:v>157</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="D23" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="F23" s="3" t="s">
         <x:v>166</x:v>
-      </x:c>
-      <x:c r="C23" s="9" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="D23" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E23" s="2" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="F23" s="3" t="s">
-        <x:v>169</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="16.5" customHeight="1">
       <x:c r="A24" s="3" t="s">
-        <x:v>157</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="s">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="F24" s="3" t="s">
         <x:v>166</x:v>
-      </x:c>
-      <x:c r="C24" s="9" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="D24" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E24" s="2" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="F24" s="3" t="s">
-        <x:v>169</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="16.5" customHeight="1">
       <x:c r="A25" s="3" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
-        <x:v>172</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="C25" s="2" t="s">
-        <x:v>173</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="D25" s="25" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="E25" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
-        <x:v>175</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="16.5" customHeight="1">
       <x:c r="A26" s="3" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
-        <x:v>176</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C26" s="2" t="s">
-        <x:v>177</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="D26" s="25" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E26" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
-        <x:v>175</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="16.5" customHeight="1">
       <x:c r="A27" s="3" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B27" s="3" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="s">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="D27" s="25" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="B27" s="3" t="s">
-        <x:v>178</x:v>
-      </x:c>
-      <x:c r="C27" s="2" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="D27" s="25" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="E27" s="2" t="s">
-        <x:v>174</x:v>
-      </x:c>
       <x:c r="F27" s="3" t="s">
-        <x:v>175</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="16.5" customHeight="1">
       <x:c r="A28" s="3" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B28" s="3" t="s">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="D28" s="25" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="B28" s="3" t="s">
-        <x:v>181</x:v>
-      </x:c>
-      <x:c r="C28" s="2" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="D28" s="25" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="E28" s="2" t="s">
-        <x:v>174</x:v>
-      </x:c>
       <x:c r="F28" s="3" t="s">
-        <x:v>175</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="16.5" customHeight="1">
       <x:c r="A29" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
-        <x:v>184</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C29" s="2" t="s">
-        <x:v>185</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="D29" s="25" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="E29" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
-        <x:v>186</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="16.5" customHeight="1">
       <x:c r="A30" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="s">
         <x:v>184</x:v>
-      </x:c>
-      <x:c r="C30" s="2" t="s">
-        <x:v>187</x:v>
       </x:c>
       <x:c r="D30" s="25" t="s">
         <x:v>18</x:v>
       </x:c>
       <x:c r="E30" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
-        <x:v>186</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="16.5" customHeight="1">
       <x:c r="A31" s="13" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
-        <x:v>184</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C31" s="2" t="s">
-        <x:v>188</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="D31" s="25" t="s">
-        <x:v>189</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="E31" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
-        <x:v>186</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="16.5" customHeight="1">
       <x:c r="A32" s="3" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B32" s="3" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="D32" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="F32" s="3" t="s">
         <x:v>190</x:v>
-      </x:c>
-      <x:c r="B32" s="3" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="C32" s="2" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="D32" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E32" s="2" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="F32" s="3" t="s">
-        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="16.5" customHeight="1">
       <x:c r="A33" s="3" t="s">
-        <x:v>194</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
-        <x:v>194</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>195</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D33" s="26" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E33" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
-        <x:v>194</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="16.5" customHeight="1">
       <x:c r="A34" s="24" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="B34" s="24" t="s">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="C34" s="27" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="D34" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E34" s="2" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="F34" s="24" t="s">
         <x:v>196</x:v>
-      </x:c>
-      <x:c r="B34" s="24" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="C34" s="27" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="D34" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E34" s="2" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="F34" s="24" t="s">
-        <x:v>199</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="16.5" customHeight="1">
       <x:c r="A35" s="3" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B35" s="3" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="C35" s="3" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D35" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E35" s="3" t="s">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="B35" s="3" t="s">
+      <x:c r="F35" s="3" t="s">
         <x:v>201</x:v>
-      </x:c>
-      <x:c r="C35" s="3" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="D35" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E35" s="3" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="F35" s="3" t="s">
-        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="16.5" customHeight="1">
       <x:c r="A36" s="3" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B36" s="3" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="D36" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E36" s="3" t="s">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="B36" s="3" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="C36" s="3" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="D36" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E36" s="3" t="s">
-        <x:v>203</x:v>
-      </x:c>
       <x:c r="F36" s="3" t="s">
-        <x:v>207</x:v>
+        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="16.5" customHeight="1">
       <x:c r="A37" s="3" t="s">
-        <x:v>200</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
-        <x:v>201</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>208</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="D37" s="26" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>209</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
-        <x:v>210</x:v>
+        <x:v>207</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="16.5" customHeight="1">
       <x:c r="A38" s="3" t="s">
-        <x:v>200</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B38" s="23" t="s">
-        <x:v>205</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C38" s="23" t="s">
-        <x:v>211</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="D38" s="26" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="F38" s="3" t="s">
         <x:v>209</x:v>
-      </x:c>
-      <x:c r="F38" s="3" t="s">
-        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="39" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A39" s="3" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="C39" s="3" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="D39" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E39" s="2" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="s">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="B39" s="3" t="s">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="C39" s="3" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="D39" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E39" s="2" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="F39" s="3" t="s">
-        <x:v>216</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="16.5" customHeight="1">
       <x:c r="A40" s="3" t="s">
-        <x:v>213</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="B40" s="3" t="s">
-        <x:v>217</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="C40" s="3" t="s">
-        <x:v>218</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="D40" s="26" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E40" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F40" s="3" t="s">
-        <x:v>219</x:v>
+        <x:v>216</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="16.5" customHeight="1">
       <x:c r="A41" s="3" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="B41" s="3" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="C41" s="2" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="D41" s="26" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E41" s="2" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="F41" s="3" t="s">
         <x:v>220</x:v>
-      </x:c>
-      <x:c r="B41" s="3" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="C41" s="2" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="D41" s="26" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E41" s="2" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="F41" s="3" t="s">
-        <x:v>223</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9014,164 +8991,164 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="s">
-        <x:v>110</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B1" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C1" s="5" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="s">
         <x:v>111</x:v>
-      </x:c>
-      <x:c r="D1" s="4" t="s">
-        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="27.600000381469727" customHeight="1">
       <x:c r="A2" s="48" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="C2" s="3" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="D2" s="3" t="s">
         <x:v>224</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="C2" s="3" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="D2" s="3" t="s">
-        <x:v>227</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="19.899999618530273" customHeight="1">
       <x:c r="A3" s="54"/>
       <x:c r="B3" s="2" t="s">
-        <x:v>228</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>229</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>230</x:v>
+        <x:v>227</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="18.600000381469727" customHeight="1">
       <x:c r="A4" s="54"/>
       <x:c r="B4" s="2" t="s">
-        <x:v>231</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>232</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>233</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="19.899999618530273" customHeight="1">
       <x:c r="A5" s="54"/>
       <x:c r="B5" s="2" t="s">
-        <x:v>234</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>235</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>236</x:v>
+        <x:v>233</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="19.899999618530273" customHeight="1">
       <x:c r="A6" s="54"/>
       <x:c r="B6" s="2" t="s">
-        <x:v>237</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>238</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>239</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="19.899999618530273" customHeight="1">
       <x:c r="A7" s="55"/>
       <x:c r="B7" s="2" t="s">
-        <x:v>240</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
-        <x:v>241</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="D7" s="2" t="s">
-        <x:v>242</x:v>
+        <x:v>239</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="48" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="s">
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="s">
         <x:v>243</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="s">
-        <x:v>244</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="D8" s="9" t="s">
-        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="54"/>
       <x:c r="B9" s="9" t="s">
-        <x:v>247</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="C9" s="9" t="s">
-        <x:v>248</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="D9" s="9" t="s">
-        <x:v>249</x:v>
+        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="54"/>
       <x:c r="B10" s="9" t="s">
-        <x:v>250</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C10" s="9" t="s">
-        <x:v>251</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D10" s="9" t="s">
-        <x:v>252</x:v>
+        <x:v>249</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="54"/>
       <x:c r="B11" s="9" t="s">
-        <x:v>253</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="C11" s="9" t="s">
-        <x:v>254</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="D11" s="9" t="s">
-        <x:v>255</x:v>
+        <x:v>252</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="54"/>
       <x:c r="B12" s="9" t="s">
-        <x:v>256</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="C12" s="9" t="s">
-        <x:v>257</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="D12" s="9" t="s">
-        <x:v>258</x:v>
+        <x:v>255</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="55"/>
       <x:c r="B13" s="9" t="s">
-        <x:v>259</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="C13" s="9" t="s">
-        <x:v>260</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="D13" s="9" t="s">
-        <x:v>261</x:v>
+        <x:v>258</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>